<commit_message>
Atualização do Otimizador de Trajetória
</commit_message>
<xml_diff>
--- a/Veiculos.xlsx
+++ b/Veiculos.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Leandro\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Leandro\Desktop\PIC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BB4D3FE7-56DA-468C-89D7-3FEC291B63BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F4DE577-D1E3-439A-98B9-D66CA51BAAE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="18737" yWindow="0" windowWidth="14263" windowHeight="17880" xr2:uid="{856E2F04-0F70-4448-8706-999C0112B3E8}"/>
+    <workbookView xWindow="13577" yWindow="591" windowWidth="19406" windowHeight="17795" xr2:uid="{856E2F04-0F70-4448-8706-999C0112B3E8}"/>
   </bookViews>
   <sheets>
     <sheet name="Folha1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>d</t>
   </si>
@@ -47,62 +47,65 @@
     <t>CD</t>
   </si>
   <si>
+    <t>m1_0</t>
+  </si>
+  <si>
+    <t>mf1</t>
+  </si>
+  <si>
+    <t>Isp1</t>
+  </si>
+  <si>
+    <t>T2W1</t>
+  </si>
+  <si>
+    <t>T1</t>
+  </si>
+  <si>
+    <t>m_flux1</t>
+  </si>
+  <si>
+    <t>m2_0</t>
+  </si>
+  <si>
+    <t>mf2</t>
+  </si>
+  <si>
+    <t>Isp2</t>
+  </si>
+  <si>
+    <t>T2W2</t>
+  </si>
+  <si>
+    <t>T2</t>
+  </si>
+  <si>
+    <t>m_flux2</t>
+  </si>
+  <si>
+    <t>V1</t>
+  </si>
+  <si>
+    <t>V2</t>
+  </si>
+  <si>
+    <t>V0</t>
+  </si>
+  <si>
+    <t>h_pitchOver</t>
+  </si>
+  <si>
     <t>gg0</t>
   </si>
   <si>
-    <t>m1_0</t>
-  </si>
-  <si>
-    <t>mf1</t>
-  </si>
-  <si>
-    <t>Isp1</t>
-  </si>
-  <si>
-    <t>T2W1</t>
-  </si>
-  <si>
-    <t>T1</t>
-  </si>
-  <si>
-    <t>m_flux1</t>
-  </si>
-  <si>
-    <t>m2_0</t>
-  </si>
-  <si>
-    <t>mf2</t>
-  </si>
-  <si>
-    <t>Isp2</t>
-  </si>
-  <si>
-    <t>T2W2</t>
-  </si>
-  <si>
-    <t>T2</t>
-  </si>
-  <si>
-    <t>m_flux2</t>
-  </si>
-  <si>
-    <t>h_pitchOver</t>
-  </si>
-  <si>
-    <t>V1</t>
-  </si>
-  <si>
-    <t>V2</t>
-  </si>
-  <si>
-    <t>V3</t>
+    <t>t_sei</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -114,13 +117,6 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF27251E"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -146,7 +142,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -154,7 +150,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -489,7 +484,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54CFCF9D-CD75-497A-BB5F-76760AAC69CB}">
-  <dimension ref="A1:H46"/>
+  <dimension ref="A1:H44"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="11.4609375" customWidth="1"/>
@@ -500,10 +495,10 @@
         <v>17</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
@@ -517,6 +512,12 @@
       <c r="B2">
         <v>1.5</v>
       </c>
+      <c r="C2">
+        <v>1.5</v>
+      </c>
+      <c r="D2">
+        <v>1.5</v>
+      </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
@@ -526,6 +527,14 @@
         <f>PI()*(B2/2)^2</f>
         <v>1.7671458676442586</v>
       </c>
+      <c r="C3">
+        <f>PI()*(C2/2)^2</f>
+        <v>1.7671458676442586</v>
+      </c>
+      <c r="D3">
+        <f>PI()*(D2/2)^2</f>
+        <v>1.7671458676442586</v>
+      </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A4" s="1" t="s">
@@ -534,14 +543,25 @@
       <c r="B4">
         <v>0.2</v>
       </c>
+      <c r="C4">
+        <v>0.2</v>
+      </c>
+      <c r="D4">
+        <v>0.2</v>
+      </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="3">
-        <f>RADIANS(89.5)</f>
-        <v>1.562069680534925</v>
+      <c r="B5">
+        <v>35093.191579200073</v>
+      </c>
+      <c r="C5">
+        <v>30394.830820941643</v>
+      </c>
+      <c r="D5">
+        <v>28820.876852104713</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.4">
@@ -549,7 +569,13 @@
         <v>4</v>
       </c>
       <c r="B6">
-        <v>35093.191579200073</v>
+        <v>6031.8660951666234</v>
+      </c>
+      <c r="C6">
+        <v>5474.2373081168053</v>
+      </c>
+      <c r="D6">
+        <v>6161.3898738827074</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.4">
@@ -557,7 +583,13 @@
         <v>5</v>
       </c>
       <c r="B7">
-        <v>6031.8660951666234</v>
+        <v>302.33330000000001</v>
+      </c>
+      <c r="C7">
+        <v>302.33330000000001</v>
+      </c>
+      <c r="D7">
+        <v>302.33330000000001</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.4">
@@ -565,7 +597,13 @@
         <v>6</v>
       </c>
       <c r="B8">
-        <v>302.33330000000001</v>
+        <v>1.4</v>
+      </c>
+      <c r="C8">
+        <v>1.4</v>
+      </c>
+      <c r="D8">
+        <v>1.4</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.4">
@@ -573,7 +611,16 @@
         <v>7</v>
       </c>
       <c r="B9">
-        <v>1.4</v>
+        <f>B5*9.80665*B8</f>
+        <v>481805.30608022725</v>
+      </c>
+      <c r="C9">
+        <f>C5*9.80665*C8</f>
+        <v>417300.05473826226</v>
+      </c>
+      <c r="D9">
+        <f>D5*9.80665*D8</f>
+        <v>395690.75277436973</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.4">
@@ -581,8 +628,16 @@
         <v>8</v>
       </c>
       <c r="B10">
-        <f>B6*9.80665*B9</f>
-        <v>481805.30608022725</v>
+        <f>B9 / (B7*9.80665)</f>
+        <v>162.50432291408222</v>
+      </c>
+      <c r="C10">
+        <f>C9 / (C7*9.80665)</f>
+        <v>140.74785393907419</v>
+      </c>
+      <c r="D10">
+        <f>D9 / (D7*9.80665)</f>
+        <v>133.45942240880049</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.4">
@@ -590,8 +645,13 @@
         <v>9</v>
       </c>
       <c r="B11">
-        <f>B10 / (B8*9.80665)</f>
-        <v>162.50432291408222</v>
+        <v>3615.9909466157787</v>
+      </c>
+      <c r="C11">
+        <v>3402.5822286591219</v>
+      </c>
+      <c r="D11">
+        <v>4277.7011378106372</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.4">
@@ -599,7 +659,13 @@
         <v>10</v>
       </c>
       <c r="B12">
-        <v>3615.9909466157787</v>
+        <v>710.99307173503064</v>
+      </c>
+      <c r="C12">
+        <v>698.54067304225975</v>
+      </c>
+      <c r="D12">
+        <v>749.60386139125069</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.4">
@@ -607,7 +673,13 @@
         <v>11</v>
       </c>
       <c r="B13">
-        <v>710.99307173503064</v>
+        <v>327.33330000000001</v>
+      </c>
+      <c r="C13">
+        <v>327.33330000000001</v>
+      </c>
+      <c r="D13">
+        <v>327.33330000000001</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.4">
@@ -615,7 +687,13 @@
         <v>12</v>
       </c>
       <c r="B14">
-        <v>327.33330000000001</v>
+        <v>0.7</v>
+      </c>
+      <c r="C14">
+        <v>0.7</v>
+      </c>
+      <c r="D14">
+        <v>0.9</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.4">
@@ -623,7 +701,16 @@
         <v>13</v>
       </c>
       <c r="B15">
-        <v>0.7</v>
+        <f>B11*9.80665*B14</f>
+        <v>24822.530331640737</v>
+      </c>
+      <c r="C15">
+        <f>C11*9.80665*C14</f>
+        <v>23357.553108875982</v>
+      </c>
+      <c r="D15">
+        <f>D11*9.80665*D14</f>
+        <v>37754.926076799617</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.4">
@@ -631,67 +718,100 @@
         <v>14</v>
       </c>
       <c r="B16">
-        <f>B12*9.80665*B15</f>
-        <v>24822.530331640737</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.4">
+        <f>B15 / (B13*9.80665)</f>
+        <v>7.732771650886253</v>
+      </c>
+      <c r="C16">
+        <f>C15 / (C13*9.80665)</f>
+        <v>7.2763985823055126</v>
+      </c>
+      <c r="D16">
+        <f>D15 / (D13*9.80665)</f>
+        <v>11.761501271118989</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A17" s="1" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B17">
-        <f>B16 / (B14*9.80665)</f>
-        <v>7.732771650886253</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.4">
+        <v>199</v>
+      </c>
+      <c r="C17">
+        <v>201</v>
+      </c>
+      <c r="D17">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A18" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B18">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A19" s="1"/>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.4">
+        <f>RADIANS(89.5)</f>
+        <v>1.562069680534925</v>
+      </c>
+      <c r="C18">
+        <f>RADIANS(89.3)</f>
+        <v>1.5585790220309363</v>
+      </c>
+      <c r="D18">
+        <f>RADIANS(88.9)</f>
+        <v>1.551597705022959</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A19" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B19">
+        <v>100</v>
+      </c>
+      <c r="C19">
+        <v>2</v>
+      </c>
+      <c r="D19">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A20" s="1"/>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A21" s="1"/>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A22" s="1"/>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A23" s="1"/>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A24" s="1"/>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A25" s="1"/>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A26" s="1"/>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A27" s="1"/>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A28" s="1"/>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A29" s="1"/>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A30" s="1"/>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A31" s="1"/>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A32" s="1"/>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.4">
@@ -716,10 +836,10 @@
       <c r="A39" s="1"/>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.4">
-      <c r="A40" s="1"/>
+      <c r="A40" s="2"/>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.4">
-      <c r="A41" s="1"/>
+      <c r="A41" s="2"/>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A42" s="2"/>
@@ -729,12 +849,6 @@
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A44" s="2"/>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.4">
-      <c r="A45" s="2"/>
-    </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.4">
-      <c r="A46" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
6DoF - Integração Física
</commit_message>
<xml_diff>
--- a/Veiculos.xlsx
+++ b/Veiculos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Leandro\Desktop\PIC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5418346-B88A-4272-BEFF-A53AB3B1B2F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEA08D90-40D6-46B6-A7B3-34B5F548842B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16406" yWindow="0" windowWidth="16594" windowHeight="17880" xr2:uid="{856E2F04-0F70-4448-8706-999C0112B3E8}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{856E2F04-0F70-4448-8706-999C0112B3E8}"/>
   </bookViews>
   <sheets>
     <sheet name="Folha1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
   <si>
     <t>d</t>
   </si>
@@ -153,6 +153,21 @@
   </si>
   <si>
     <t>m_LOX_S2</t>
+  </si>
+  <si>
+    <t>ms1</t>
+  </si>
+  <si>
+    <t>ms2</t>
+  </si>
+  <si>
+    <t>mPL</t>
+  </si>
+  <si>
+    <t>h_S1</t>
+  </si>
+  <si>
+    <t>h_S2</t>
   </si>
 </sst>
 </file>
@@ -201,9 +216,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -538,7 +551,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54CFCF9D-CD75-497A-BB5F-76760AAC69CB}">
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:H71"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="12.4609375" customWidth="1"/>
@@ -575,7 +588,7 @@
         <v>1.5</v>
       </c>
       <c r="E2">
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.4">
@@ -596,7 +609,7 @@
       </c>
       <c r="E3">
         <f>PI()*(E2/2)^2</f>
-        <v>1.7671458676442586</v>
+        <v>2.2698006922186251</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.4">
@@ -1035,25 +1048,135 @@
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A37" s="1"/>
+      <c r="A37" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E37">
+        <v>1883.6887360720702</v>
+      </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A38" s="1"/>
+      <c r="A38" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E38">
+        <v>249.6038614</v>
+      </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A39" s="2"/>
+      <c r="A39" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E39">
+        <v>500</v>
+      </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A40" s="2"/>
+      <c r="A40" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E40">
+        <v>12.765200767150406</v>
+      </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A41" s="2"/>
+      <c r="A41" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E41">
+        <f>3.4+2.59829862446971</f>
+        <v>5.9982986244697098</v>
+      </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A42" s="2"/>
+      <c r="A42" s="1"/>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A43" s="2"/>
+      <c r="A43" s="1"/>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A44" s="2"/>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A45" s="2"/>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A46" s="2"/>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A47" s="2"/>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A48" s="2"/>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A49" s="2"/>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A50" s="2"/>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A51" s="2"/>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A52" s="2"/>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A53" s="2"/>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A54" s="2"/>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A55" s="2"/>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A56" s="2"/>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A57" s="2"/>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A58" s="2"/>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A59" s="2"/>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A60" s="2"/>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A61" s="2"/>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A62" s="2"/>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A63" s="2"/>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A64" s="2"/>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A65" s="2"/>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A66" s="2"/>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A67" s="2"/>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A68" s="2"/>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A69" s="2"/>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A70" s="2"/>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.4">
+      <c r="A71" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>